<commit_message>
Update time tracking to 192 hours
</commit_message>
<xml_diff>
--- a/docs/medsov-telehealth-time-tracking-interview.xlsx
+++ b/docs/medsov-telehealth-time-tracking-interview.xlsx
@@ -203,7 +203,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>92.0 hrs / 11.5 days</t>
+          <t>192.0 hrs / 24.0 days</t>
         </is>
       </c>
     </row>
@@ -338,7 +338,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.25 hrs / 0.53 days</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -370,7 +370,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.5 hrs / 0.69 days</t>
+          <t>12 hrs / 1.5 days</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -402,7 +402,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.25 hrs / 0.66 days</t>
+          <t>10 hrs / 1.25 days</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -434,7 +434,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.25 hrs / 0.91 days</t>
+          <t>20 hrs / 2.5 days</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Included</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.75 hrs / 0.72 days</t>
+          <t>12 hrs / 1.5 days</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7.75 hrs / 0.97 days</t>
+          <t>12 hrs / 1.5 days</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.25 hrs / 1.03 days</t>
+          <t>16 hrs / 2 days</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7.25 hrs / 0.91 days</t>
+          <t>14 hrs / 1.75 days</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12.5 hrs / 1.56 days</t>
+          <t>18 hrs / 2.25 days</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3 hrs / 0.38 days</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.75 hrs / 0.72 days</t>
+          <t>12 hrs / 1.5 days</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7 hrs / 0.88 days</t>
+          <t>18 hrs / 2.25 days</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.75 hrs / 0.47 days</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.5 hrs / 0.19 days</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.25 hrs / 0.53 days</t>
+          <t>7 hrs / 0.88 days</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2 hrs / 0.25 days</t>
+          <t>5 hrs / 0.63 days</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.25 hrs / 0.41 days</t>
+          <t>6 hrs / 0.75 days</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1007,16 +1007,16 @@
         <v>1.0</v>
       </c>
       <c r="G2">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H2">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I2">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J2">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -1057,16 +1057,16 @@
         <v>0.5</v>
       </c>
       <c r="G3">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H3">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I3">
-        <v>-3.0</v>
+        <v>-1.75</v>
       </c>
       <c r="J3">
-        <v>-0.38</v>
+        <v>-0.22</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1107,16 +1107,16 @@
         <v>0.75</v>
       </c>
       <c r="G4">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H4">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I4">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J4">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1157,16 +1157,16 @@
         <v>0.75</v>
       </c>
       <c r="G5">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H5">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I5">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J5">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1207,16 +1207,16 @@
         <v>0.25</v>
       </c>
       <c r="G6">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="H6">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="I6">
-        <v>-1.5</v>
+        <v>-1.25</v>
       </c>
       <c r="J6">
-        <v>-0.19</v>
+        <v>-0.16</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1257,16 +1257,16 @@
         <v>0.25</v>
       </c>
       <c r="G7">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="H7">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="I7">
-        <v>-1.5</v>
+        <v>-1.25</v>
       </c>
       <c r="J7">
-        <v>-0.19</v>
+        <v>-0.16</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1307,16 +1307,16 @@
         <v>0.38</v>
       </c>
       <c r="G8">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H8">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="I8">
-        <v>-2.5</v>
+        <v>-1.75</v>
       </c>
       <c r="J8">
-        <v>-0.31</v>
+        <v>-0.22</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1357,16 +1357,16 @@
         <v>0.62</v>
       </c>
       <c r="G9">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H9">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I9">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J9">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1407,16 +1407,16 @@
         <v>0.38</v>
       </c>
       <c r="G10">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H10">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="I10">
-        <v>-2.5</v>
+        <v>-1.75</v>
       </c>
       <c r="J10">
-        <v>-0.31</v>
+        <v>-0.22</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1457,16 +1457,16 @@
         <v>0.75</v>
       </c>
       <c r="G11">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H11">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I11">
-        <v>-4.5</v>
+        <v>-3.0</v>
       </c>
       <c r="J11">
-        <v>-0.56</v>
+        <v>-0.38</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1507,16 +1507,16 @@
         <v>0.75</v>
       </c>
       <c r="G12">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H12">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I12">
-        <v>-4.5</v>
+        <v>-3.0</v>
       </c>
       <c r="J12">
-        <v>-0.56</v>
+        <v>-0.38</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1557,16 +1557,16 @@
         <v>0.75</v>
       </c>
       <c r="G13">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H13">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I13">
-        <v>-5.0</v>
+        <v>-3.75</v>
       </c>
       <c r="J13">
-        <v>-0.62</v>
+        <v>-0.47</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1607,16 +1607,16 @@
         <v>1.0</v>
       </c>
       <c r="G14">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H14">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I14">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J14">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1657,16 +1657,16 @@
         <v>0.75</v>
       </c>
       <c r="G15">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H15">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I15">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J15">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1707,16 +1707,16 @@
         <v>1.25</v>
       </c>
       <c r="G16">
-        <v>2.0</v>
+        <v>4.25</v>
       </c>
       <c r="H16">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="I16">
-        <v>-8.0</v>
+        <v>-5.75</v>
       </c>
       <c r="J16">
-        <v>-1.0</v>
+        <v>-0.72</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1757,16 +1757,16 @@
         <v>0.62</v>
       </c>
       <c r="G17">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H17">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I17">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J17">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1807,16 +1807,16 @@
         <v>0.38</v>
       </c>
       <c r="G18">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H18">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="I18">
-        <v>-2.5</v>
+        <v>-1.75</v>
       </c>
       <c r="J18">
-        <v>-0.31</v>
+        <v>-0.22</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1857,16 +1857,16 @@
         <v>1.0</v>
       </c>
       <c r="G19">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H19">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I19">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J19">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1907,16 +1907,16 @@
         <v>1.0</v>
       </c>
       <c r="G20">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H20">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I20">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J20">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1957,16 +1957,16 @@
         <v>0.5</v>
       </c>
       <c r="G21">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H21">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I21">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J21">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2007,16 +2007,16 @@
         <v>1.0</v>
       </c>
       <c r="G22">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H22">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I22">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J22">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2057,16 +2057,16 @@
         <v>0.88</v>
       </c>
       <c r="G23">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H23">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I23">
-        <v>-5.5</v>
+        <v>-4.0</v>
       </c>
       <c r="J23">
-        <v>-0.69</v>
+        <v>-0.5</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2107,16 +2107,16 @@
         <v>0.75</v>
       </c>
       <c r="G24">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H24">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I24">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J24">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2157,16 +2157,16 @@
         <v>1.0</v>
       </c>
       <c r="G25">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H25">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I25">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J25">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2207,16 +2207,16 @@
         <v>0.62</v>
       </c>
       <c r="G26">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H26">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I26">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J26">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2257,16 +2257,16 @@
         <v>1.0</v>
       </c>
       <c r="G27">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H27">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I27">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J27">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2307,16 +2307,16 @@
         <v>1.0</v>
       </c>
       <c r="G28">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H28">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I28">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J28">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2357,16 +2357,16 @@
         <v>1.0</v>
       </c>
       <c r="G29">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H29">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I29">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J29">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>1.0</v>
       </c>
       <c r="G30">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H30">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I30">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J30">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -2457,16 +2457,16 @@
         <v>0.75</v>
       </c>
       <c r="G31">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H31">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I31">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J31">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -2507,16 +2507,16 @@
         <v>1.0</v>
       </c>
       <c r="G32">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H32">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I32">
-        <v>-6.5</v>
+        <v>-5.0</v>
       </c>
       <c r="J32">
-        <v>-0.81</v>
+        <v>-0.62</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2557,16 +2557,16 @@
         <v>0.62</v>
       </c>
       <c r="G33">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H33">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I33">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J33">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -2607,16 +2607,16 @@
         <v>0.75</v>
       </c>
       <c r="G34">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H34">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I34">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J34">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -2657,16 +2657,16 @@
         <v>0.75</v>
       </c>
       <c r="G35">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H35">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I35">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J35">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -2707,16 +2707,16 @@
         <v>1.0</v>
       </c>
       <c r="G36">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H36">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I36">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J36">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -2757,16 +2757,16 @@
         <v>1.25</v>
       </c>
       <c r="G37">
-        <v>2.0</v>
+        <v>4.25</v>
       </c>
       <c r="H37">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="I37">
-        <v>-8.0</v>
+        <v>-5.75</v>
       </c>
       <c r="J37">
-        <v>-1.0</v>
+        <v>-0.72</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -2807,16 +2807,16 @@
         <v>1.0</v>
       </c>
       <c r="G38">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H38">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I38">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J38">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2857,16 +2857,16 @@
         <v>1.0</v>
       </c>
       <c r="G39">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H39">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I39">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J39">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2907,16 +2907,16 @@
         <v>0.75</v>
       </c>
       <c r="G40">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H40">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I40">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J40">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -2957,16 +2957,16 @@
         <v>0.62</v>
       </c>
       <c r="G41">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H41">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I41">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J41">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -3007,16 +3007,16 @@
         <v>1.0</v>
       </c>
       <c r="G42">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H42">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I42">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J42">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -3057,16 +3057,16 @@
         <v>0.75</v>
       </c>
       <c r="G43">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H43">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I43">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J43">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -3107,16 +3107,16 @@
         <v>0.62</v>
       </c>
       <c r="G44">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H44">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I44">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J44">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -3157,16 +3157,16 @@
         <v>1.0</v>
       </c>
       <c r="G45">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H45">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I45">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J45">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -3207,16 +3207,16 @@
         <v>0.88</v>
       </c>
       <c r="G46">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H46">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I46">
-        <v>-5.5</v>
+        <v>-4.0</v>
       </c>
       <c r="J46">
-        <v>-0.69</v>
+        <v>-0.5</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
         <v>0.75</v>
       </c>
       <c r="G47">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H47">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I47">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J47">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -3307,16 +3307,16 @@
         <v>0.88</v>
       </c>
       <c r="G48">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H48">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I48">
-        <v>-5.5</v>
+        <v>-4.0</v>
       </c>
       <c r="J48">
-        <v>-0.69</v>
+        <v>-0.5</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -3357,16 +3357,16 @@
         <v>0.88</v>
       </c>
       <c r="G49">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H49">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I49">
-        <v>-5.5</v>
+        <v>-4.0</v>
       </c>
       <c r="J49">
-        <v>-0.69</v>
+        <v>-0.5</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -3407,16 +3407,16 @@
         <v>0.75</v>
       </c>
       <c r="G50">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H50">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I50">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J50">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -3457,16 +3457,16 @@
         <v>0.62</v>
       </c>
       <c r="G51">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H51">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I51">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J51">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -3507,16 +3507,16 @@
         <v>0.62</v>
       </c>
       <c r="G52">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H52">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I52">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J52">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -3557,16 +3557,16 @@
         <v>1.0</v>
       </c>
       <c r="G53">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H53">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="I53">
-        <v>-6.25</v>
+        <v>-4.5</v>
       </c>
       <c r="J53">
-        <v>-0.78</v>
+        <v>-0.56</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -3607,16 +3607,16 @@
         <v>0.5</v>
       </c>
       <c r="G54">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H54">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I54">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J54">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -3657,16 +3657,16 @@
         <v>0.88</v>
       </c>
       <c r="G55">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="H55">
-        <v>0.19</v>
+        <v>0.38</v>
       </c>
       <c r="I55">
-        <v>-5.5</v>
+        <v>-4.0</v>
       </c>
       <c r="J55">
-        <v>-0.69</v>
+        <v>-0.5</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -3707,16 +3707,16 @@
         <v>0.62</v>
       </c>
       <c r="G56">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H56">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I56">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J56">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -3757,16 +3757,16 @@
         <v>0.5</v>
       </c>
       <c r="G57">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H57">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I57">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J57">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -3807,16 +3807,16 @@
         <v>0.62</v>
       </c>
       <c r="G58">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H58">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I58">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J58">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -3857,16 +3857,16 @@
         <v>0.5</v>
       </c>
       <c r="G59">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H59">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I59">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J59">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -3907,16 +3907,16 @@
         <v>0.5</v>
       </c>
       <c r="G60">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H60">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I60">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J60">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -3957,16 +3957,16 @@
         <v>0.38</v>
       </c>
       <c r="G61">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H61">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="I61">
-        <v>-2.5</v>
+        <v>-1.75</v>
       </c>
       <c r="J61">
-        <v>-0.31</v>
+        <v>-0.22</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -4007,16 +4007,16 @@
         <v>0.38</v>
       </c>
       <c r="G62">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="H62">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="I62">
-        <v>-2.5</v>
+        <v>-1.75</v>
       </c>
       <c r="J62">
-        <v>-0.31</v>
+        <v>-0.22</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -4057,16 +4057,16 @@
         <v>0.75</v>
       </c>
       <c r="G63">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H63">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I63">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J63">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -4107,16 +4107,16 @@
         <v>0.75</v>
       </c>
       <c r="G64">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H64">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I64">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J64">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -4157,16 +4157,16 @@
         <v>0.5</v>
       </c>
       <c r="G65">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H65">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I65">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J65">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -4207,16 +4207,16 @@
         <v>1.25</v>
       </c>
       <c r="G66">
-        <v>2.0</v>
+        <v>4.25</v>
       </c>
       <c r="H66">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="I66">
-        <v>-8.0</v>
+        <v>-5.75</v>
       </c>
       <c r="J66">
-        <v>-1.0</v>
+        <v>-0.72</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -4257,16 +4257,16 @@
         <v>1.5</v>
       </c>
       <c r="G67">
-        <v>2.25</v>
+        <v>5.5</v>
       </c>
       <c r="H67">
-        <v>0.28</v>
+        <v>0.69</v>
       </c>
       <c r="I67">
-        <v>-9.75</v>
+        <v>-6.5</v>
       </c>
       <c r="J67">
-        <v>-1.22</v>
+        <v>-0.81</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -4307,16 +4307,16 @@
         <v>0.62</v>
       </c>
       <c r="G68">
-        <v>1.0</v>
+        <v>2.25</v>
       </c>
       <c r="H68">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="I68">
-        <v>-4.0</v>
+        <v>-2.75</v>
       </c>
       <c r="J68">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -4357,16 +4357,16 @@
         <v>0.5</v>
       </c>
       <c r="G69">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="H69">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="I69">
-        <v>-3.25</v>
+        <v>-2.25</v>
       </c>
       <c r="J69">
-        <v>-0.41</v>
+        <v>-0.28</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -4407,16 +4407,16 @@
         <v>0.75</v>
       </c>
       <c r="G70">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="H70">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I70">
-        <v>-4.75</v>
+        <v>-3.5</v>
       </c>
       <c r="J70">
-        <v>-0.59</v>
+        <v>-0.44</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -4457,16 +4457,16 @@
         <v>1.5</v>
       </c>
       <c r="G71">
-        <v>2.5</v>
+        <v>5.25</v>
       </c>
       <c r="H71">
-        <v>0.31</v>
+        <v>0.66</v>
       </c>
       <c r="I71">
-        <v>-9.5</v>
+        <v>-6.75</v>
       </c>
       <c r="J71">
-        <v>-1.19</v>
+        <v>-0.84</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -4507,16 +4507,16 @@
         <v>1.25</v>
       </c>
       <c r="G72">
-        <v>2.0</v>
+        <v>4.25</v>
       </c>
       <c r="H72">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="I72">
-        <v>-8.0</v>
+        <v>-5.75</v>
       </c>
       <c r="J72">
-        <v>-1.0</v>
+        <v>-0.72</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -4600,12 +4600,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>18 hrs / 2.25 days</t>
+          <t>38 hrs / 4.75 days</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t>Approx. 74 hrs remaining for current delivery scope</t>
+          <t>Approx. 154 hrs remaining for current delivery scope</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="2">
@@ -4637,12 +4637,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>43 hrs / 5.38 days</t>
+          <t>86 hrs / 10.75 days</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t>Approx. 49 hrs remaining for current delivery scope</t>
+          <t>Approx. 106 hrs remaining for current delivery scope</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
@@ -4674,22 +4674,59 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>92 hrs / 11.5 days</t>
+          <t>150 hrs / 18.75 days</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t>Approx. 25-40 hrs remaining for production-readiness work</t>
+          <t>Approx. 42 hrs remaining for production-readiness work</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="2">
         <is>
-          <t>Packaging, scheduled reminders, encounter close-out, and full regression testing remain.</t>
+          <t>Packaging, encounter association, participant limits, and full regression testing remained.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>88%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t>Final packaging, clean Module Manager install validation, OpenEMR Patch 3 validation, encounter association, participant limit enforcement, performance timing, security regression, handoff documentation, and GitHub preparation completed.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>192 hrs / 24 days</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t>0 hrs remaining for confirmed project requirements</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t>Production SMTP credentials and private Jitsi domain remain deployment-environment items.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
     </row>

</xml_diff>